<commit_message>
Add documented pytest coverage and case statuses
</commit_message>
<xml_diff>
--- a/phon_book/docs/TEST_CASES.xlsx
+++ b/phon_book/docs/TEST_CASES.xlsx
@@ -4,26 +4,41 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
+      <charset val="1"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="0"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,19 +58,39 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="6">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -128,41 +163,41 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -170,375 +205,272 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:tint val="15000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:shade val="51000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
                 <a:shade val="93000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="94000"/>
-                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="20000"/>
-                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="30000"/>
-                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:O36"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" style="2" min="1" max="1"/>
+    <col width="21" customWidth="1" style="2" min="2" max="3"/>
+    <col width="48" customWidth="1" style="2" min="4" max="9"/>
+    <col width="15" customWidth="1" style="2" min="10" max="10"/>
+    <col width="14" customWidth="1" style="2" min="11" max="11"/>
+    <col width="18" customWidth="1" style="2" min="12" max="12"/>
+    <col width="14" customWidth="1" style="2" min="13" max="13"/>
+    <col width="21" customWidth="1" style="2" min="14" max="14"/>
+    <col width="48" customWidth="1" style="2" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="3">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Related Scenario ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Execution Mode</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Notes / Evidence</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="2" ht="82.05" customHeight="1" s="3">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>TC-001</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>SCN-003</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Validate login by email requirement mismatch</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Verify whether a registered user can authenticate using email and password as required by the assignment.</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database; no active dependency failure.</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>User A: username=amir, email=amir@example.com, password=1234</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register user amir with email amir@example.com and password 1234.
@@ -546,74 +478,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>System should support login by email or return a controlled requirement-mismatch outcome without server termination.</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Email-based login is not supported; server stops instead of returning a controlled success/failure flow.</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L2" s="1" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M2" s="1" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="N2" s="1" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns plain string not-found error and terminates server.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+    <row r="3" ht="55.2" customHeight="1" s="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>TC-002</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>SCN-005</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Reject duplicate email registration</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Verify that two different accounts cannot register with the same email address.</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>User A: username=user_a, email=same@example.com, password=1234; User B: username=user_b, email=same@example.com, password=1234</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register User A.
@@ -621,74 +558,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Second registration should be rejected cleanly, server should remain running, and response should be structured.</t>
         </is>
       </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K3" s="1" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Duplicate email registration was accepted; second user was created successfully.</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L3" s="1" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M3" s="1" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently allows duplicate email registration.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+    <row r="4" ht="55.2" customHeight="1" s="3">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>TC-003</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>SCN-004</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Reject duplicate username without crashing server</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Verify that duplicate username registration is handled as a controlled validation error.</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>User A: username=dup, email=dup1@example.com, password=1234; User B: username=dup, email=dup2@example.com, password=1234</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register User A.
@@ -696,296 +638,316 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Second registration should be rejected with a structured validation result and server should continue running.</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Duplicate username path did not return a controlled structured validation error; server did not behave as expected.</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L4" s="1" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M4" s="1" t="inlineStr">
+      <c r="N4" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N4" s="1" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns raw UNIQUE constraint text and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="5" ht="41.75" customHeight="1" s="3">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>TC-004</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>SCN-027</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Handle missing signup username safely</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Verify that signup with a missing username field does not crash the server.</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Signup payload missing username; password=1234; email=m@example.com</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send sign_up request without username.
 3. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled validation error and keep the server alive.</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Missing signup username did not return a controlled validation response; server stopped.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L5" s="1" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M5" s="1" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N5" s="1" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns KeyError text and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+    <row r="6" ht="41.75" customHeight="1" s="3">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>TC-005</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>SCN-029</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Handle non-string password safely during signup</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Verify that invalid password data type is validated before hashing logic executes.</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Signup payload: username=typed, password=1234 as integer, email=typed@example.com</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send sign_up request with integer password.
 3. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>System should reject the input cleanly without raw exception output or server termination.</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K6" s="1" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Non-string password did not return a controlled validation response; server stopped.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L6" s="1" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M6" s="1" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N6" s="1" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently raises AttributeError and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="7" ht="55.2" customHeight="1" s="3">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TC-006</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>SCN-028</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Handle missing phone number safely on contact creation</t>
         </is>
       </c>
-      <c r="D7" s="1" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Verify that add_phone_user with missing phone_number does not crash the server.</t>
         </is>
       </c>
-      <c r="E7" s="1" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database or schema initialized.</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Contact payload: username=ali with no phone_number</t>
         </is>
       </c>
-      <c r="G7" s="1" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send add_phone_user request without phone_number.
 3. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H7" s="1" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled validation error and keep the server alive.</t>
         </is>
       </c>
-      <c r="I7" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K7" s="1" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>After satisfying auth prerequisites, missing phone_number still did not return a controlled structured validation response; server stopped.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L7" s="1" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M7" s="1" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N7" s="1" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns KeyError text and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+    <row r="8" ht="55.2" customHeight="1" s="3">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>TC-007</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>SCN-009</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Block contact creation before authentication</t>
         </is>
       </c>
-      <c r="D8" s="1" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Verify whether add_phone_user is denied when no sign_in has been performed.</t>
         </is>
       </c>
-      <c r="E8" s="1" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialization path is known or completed; no active authenticated session.</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Contact payload: username=ali, phone_number=12092</t>
         </is>
       </c>
-      <c r="G8" s="1" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure no sign_in command is sent.
@@ -993,74 +955,79 @@
 4. Observe reply and whether contact is created.</t>
         </is>
       </c>
-      <c r="H8" s="1" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>System should reject the request as unauthorized if authentication is required.</t>
         </is>
       </c>
-      <c r="I8" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J8" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K8" s="1" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Contact creation after sign_up but without sign_in was still allowed instead of being blocked by authorization.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="L8" s="1" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M8" s="1" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N8" s="1" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently allows contact creation once schema exists.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+    <row r="9" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>TC-008</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>SCN-010</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Block contact list retrieval before authentication</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Verify whether get_all_phone_users is denied without prior sign_in.</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; at least one contact exists.</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Request payload: get_all_phone_users with empty parameters</t>
         </is>
       </c>
-      <c r="G9" s="1" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure schema exists and at least one contact is present.
@@ -1068,148 +1035,158 @@
 4. Observe reply.</t>
         </is>
       </c>
-      <c r="H9" s="1" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>System should reject the request as unauthorized if authentication is required.</t>
         </is>
       </c>
-      <c r="I9" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J9" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K9" s="1" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Contact list retrieval without sign_in was still allowed after data setup instead of being blocked by authorization.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="L9" s="1" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M9" s="1" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N9" s="1" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently allows unauthenticated list retrieval after schema initialization.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+    <row r="10" ht="41.75" customHeight="1" s="3">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>TC-009</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>SCN-032</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Return documented success response structure</t>
         </is>
       </c>
-      <c r="D10" s="1" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Verify that successful command execution returns the documented command_name/result structure.</t>
         </is>
       </c>
-      <c r="E10" s="1" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Valid sign_up or contact-creation request batch</t>
         </is>
       </c>
-      <c r="G10" s="1" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send a valid successful command batch.
 3. Inspect the reply structure.</t>
         </is>
       </c>
-      <c r="H10" s="1" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Each successful result item should include command_name and result in structured form.</t>
         </is>
       </c>
-      <c r="I10" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J10" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K10" s="1" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Successful command execution returned a structured reply containing command_name and result.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
       </c>
-      <c r="L10" s="1" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M10" s="1" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N10" s="1" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Success path was observed to be structured during validation.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="11" ht="55.2" customHeight="1" s="3">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>TC-010</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>SCN-033</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Return structured error for duplicate username failure</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Verify that expected business-rule failures return structured error results instead of raw DB messages.</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Duplicate-username signup sequence using username=dup</t>
         </is>
       </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register username dup once.
@@ -1217,74 +1194,79 @@
 4. Inspect reply structure and server stability.</t>
         </is>
       </c>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>System should return a structured error result, should not expose DB internals, and should remain running.</t>
         </is>
       </c>
-      <c r="I11" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K11" s="1" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Duplicate username failure did not return a structured error and the server did not remain alive.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Contract</t>
         </is>
       </c>
-      <c r="L11" s="1" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M11" s="1" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N11" s="1" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns raw UNIQUE constraint text and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="12" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>TC-011</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>SCN-034</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Keep server alive after invalid auth request</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Verify service resilience after an invalid authentication request.</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Invalid signup payload missing username</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send invalid signup request missing username.
@@ -1292,222 +1274,237 @@
 4. Observe whether server still processes the second request.</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Server should survive the invalid request and process subsequent valid requests normally.</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K12" s="1" t="inlineStr">
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Invalid request still caused server termination instead of resilient continued service.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
       </c>
-      <c r="L12" s="1" t="inlineStr">
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M12" s="1" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently terminates server after the invalid request.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="13" ht="41.75" customHeight="1" s="3">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>TC-012</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>SCN-035</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Avoid leaking traceback and SQL details in error replies</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Verify that error paths do not expose internal implementation details to the client.</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database.</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>A failure-producing request such as duplicate signup or missing contact add_phone_number</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Trigger a controlled failure.
 3. Inspect client-visible reply and server-visible output.</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Error output should be controlled and should not expose tracebacks, SQL statements, or model internals.</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K13" s="1" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Failure paths still leak internal details instead of controlled safe error output.</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="L13" s="1" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M13" s="1" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="N13" s="1" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently leaks traceback and SQL/model details.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="14" ht="55.2" customHeight="1" s="3">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>TC-013</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>SCN-036</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Initialize phonebook schema before first contact operation</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Verify that the first phonebook operation on a clean database succeeds without requiring a prior auth command.</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database with no prior auth operation.</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Request payload: add_phone_user username=ali, phone_number=12092</t>
         </is>
       </c>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>1. Start server on a clean database.
 2. Send add_phone_user as the first DB-touching command.
 3. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>System should create any required tables or otherwise support the command without raw OperationalError.</t>
         </is>
       </c>
-      <c r="I14" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K14" s="1" t="inlineStr">
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>After satisfying auth prerequisites on a clean database, the first phonebook operation succeeded and returned a structured success result.</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Data Consistency</t>
         </is>
       </c>
-      <c r="L14" s="1" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M14" s="1" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N14" s="1" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently fails with no such table: phone_user_table and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="15" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>TC-014</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>SCN-015</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Reject duplicate contact name without crashing server</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Verify that creating a contact with an existing contact name returns a controlled failure.</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database; schema initialized; contact ali already exists.</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Contact A: username=ali, phone_number=12092; duplicate contact: username=ali, phone_number=77777</t>
         </is>
       </c>
-      <c r="G15" s="1" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Initialize schema if needed.
@@ -1516,74 +1513,79 @@
 5. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>System should reject the duplicate contact with a controlled error and remain running.</t>
         </is>
       </c>
-      <c r="I15" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J15" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K15" s="1" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>After satisfying auth prerequisites, duplicate contact name still did not return a controlled rejection and server stopped.</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L15" s="1" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M15" s="1" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N15" s="1" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns raw UNIQUE constraint error and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="16" ht="82.05" customHeight="1" s="3">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>TC-015</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>SCN-016</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Reject duplicate phone number without crashing server</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Verify that reusing an existing phone number is handled as a controlled business failure.</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database; schema initialized; an existing phone number already exists.</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Contact A: username=ali, phone_number=12092; Contact B: username=reza, phone_number=12092</t>
         </is>
       </c>
-      <c r="G16" s="1" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Initialize schema if needed.
@@ -1592,74 +1594,79 @@
 5. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>System should reject the duplicate phone number with a controlled error and remain running.</t>
         </is>
       </c>
-      <c r="I16" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K16" s="1" t="inlineStr">
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>After satisfying auth prerequisites, duplicate phone number still did not return a controlled rejection and server stopped.</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L16" s="1" t="inlineStr">
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M16" s="1" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N16" s="1" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns raw UNIQUE constraint error and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="17" ht="55.2" customHeight="1" s="3">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>TC-016</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>SCN-017</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Handle add-phone-number for non-existing contact gracefully</t>
         </is>
       </c>
-      <c r="D17" s="1" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>Verify that adding a number to a non-existing contact returns a controlled not-found response.</t>
         </is>
       </c>
-      <c r="E17" s="1" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database; schema initialized; target contact does not exist.</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Payload: username=ghost, phone_number=9999</t>
         </is>
       </c>
-      <c r="G17" s="1" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Initialize schema if needed.
@@ -1667,222 +1674,237 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H17" s="1" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled not-found result without leaking internals or terminating the server.</t>
         </is>
       </c>
-      <c r="I17" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K17" s="1" t="inlineStr">
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>After satisfying auth prerequisites, adding a phone number to a missing contact still did not return a controlled not-found result and server stopped.</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L17" s="1" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M17" s="1" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N17" s="1" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>Validated runtime currently returns raw model/SQL details and terminates the server.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="18" ht="55.2" customHeight="1" s="3">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>TC-017</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>SCN-037</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Observe repeat-run behavior with persistent database state</t>
         </is>
       </c>
-      <c r="D18" s="1" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Verify how existing sab.db content affects repeated execution of the same manual flows.</t>
         </is>
       </c>
-      <c r="E18" s="1" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Database file already contains prior test data.</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Reuse a previously successful signup or contact-creation flow.</t>
         </is>
       </c>
-      <c r="G18" s="1" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>1. Run a successful flow once.
 2. Without resetting the database, run the same flow again.
 3. Observe differences in result and stability.</t>
         </is>
       </c>
-      <c r="H18" s="1" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Repeat-run behavior should be predictable and documented; failures should not be mistaken for unrelated defects.</t>
         </is>
       </c>
-      <c r="I18" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K18" s="1" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Repeat execution against the same persistent database did not produce a controlled duplicate-handling result; the second run stopped the server.</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Operational</t>
         </is>
       </c>
-      <c r="L18" s="1" t="inlineStr">
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M18" s="1" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="N18" s="1" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>This case is important for QA execution discipline even if persistence itself is expected.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="19" ht="55.2" customHeight="1" s="3">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>TC-018</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>SCN-001</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Register a new user with valid signup data</t>
         </is>
       </c>
-      <c r="D19" s="1" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Verify successful registration of a new account with valid required fields.</t>
         </is>
       </c>
-      <c r="E19" s="1" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Server is running; clean database; target username and email do not exist.</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>username=new_user; email=new_user@example.com; password=1234</t>
         </is>
       </c>
-      <c r="G19" s="1" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Send sign_up with valid username, email, and password.
 3. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H19" s="1" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>System should register the user successfully, return a structured success result, and remain running.</t>
         </is>
       </c>
-      <c r="I19" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J19" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K19" s="1" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Valid signup returned a structured success result and server stayed alive.</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L19" s="1" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M19" s="1" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N19" s="1" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>Wave 2 happy-path auth baseline.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="20" ht="55.2" customHeight="1" s="3">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>TC-019</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>SCN-002</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Authenticate a registered user with valid credentials</t>
         </is>
       </c>
-      <c r="D20" s="1" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Verify successful sign-in for an existing user using the implemented login format.</t>
         </is>
       </c>
-      <c r="E20" s="1" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Server is running; registered user exists.</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>username=amir; password=1234</t>
         </is>
       </c>
-      <c r="G20" s="1" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register user if needed.
@@ -1890,74 +1912,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H20" s="1" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>System should sign in the user successfully and return a structured success result.</t>
         </is>
       </c>
-      <c r="I20" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J20" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K20" s="1" t="inlineStr">
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Valid sign-in using implemented username flow returned structured success result and server stayed alive.</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L20" s="1" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M20" s="1" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N20" s="1" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Current implementation expects username, not email.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="21" ht="55.2" customHeight="1" s="3">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TC-020</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>SCN-007</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Handle wrong password login attempt</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Verify controlled behavior when a registered user provides the wrong password.</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Server is running; registered user exists.</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>username=amir; wrong_password=wrong123</t>
         </is>
       </c>
-      <c r="G21" s="1" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure user amir exists.
@@ -1965,74 +1992,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H21" s="1" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>System should reject the login attempt cleanly, avoid internal leakage, and remain running.</t>
         </is>
       </c>
-      <c r="I21" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J21" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K21" s="1" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Wrong-password login did not return a controlled structured rejection while keeping server alive.</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L21" s="1" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M21" s="1" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N21" s="1" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>Important to compare with requirement contract expectations.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="22" ht="55.2" customHeight="1" s="3">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>TC-021</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>SCN-008</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Logout the authenticated user successfully</t>
         </is>
       </c>
-      <c r="D22" s="1" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Verify successful logout of a user who has previously signed in.</t>
         </is>
       </c>
-      <c r="E22" s="1" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Server is running; registered user exists; user is signed in.</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>username=amir; password=1234</t>
         </is>
       </c>
-      <c r="G22" s="1" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Register and sign in user amir.
@@ -2040,74 +2072,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H22" s="1" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>System should report successful logout for the signed-in user.</t>
         </is>
       </c>
-      <c r="I22" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J22" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K22" s="1" t="inlineStr">
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Logout after successful sign-in returned structured success result and server stayed alive.</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>State Transition</t>
         </is>
       </c>
-      <c r="L22" s="1" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M22" s="1" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N22" s="1" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>Does not yet validate ownership weakness; that is covered in Wave 1.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+    <row r="23" ht="55.2" customHeight="1" s="3">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>TC-022</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>SCN-013</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Create a new contact with initial phone number</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Verify successful creation of a new phonebook contact and its first number.</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact and number do not exist.</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; phone_number=12092; explanation=friend</t>
         </is>
       </c>
-      <c r="G23" s="1" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure schema is initialized if required.
@@ -2115,74 +2152,79 @@
 4. Observe reply.</t>
         </is>
       </c>
-      <c r="H23" s="1" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>System should create the contact successfully and return a structured success result.</t>
         </is>
       </c>
-      <c r="I23" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J23" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K23" s="1" t="inlineStr">
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Authenticated contact creation with an initial phone number returned a structured success result.</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L23" s="1" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M23" s="1" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N23" s="1" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>Core phonebook happy path.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="24" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>TC-023</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>SCN-014</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Add a second phone number to an existing contact</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Verify successful addition of another phone number to an existing contact.</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; contact already exists.</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; existing_phone=12092; new_phone=44653112</t>
         </is>
       </c>
-      <c r="G24" s="1" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali with first phone number.
@@ -2190,74 +2232,79 @@
 4. Observe reply.</t>
         </is>
       </c>
-      <c r="H24" s="1" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>System should add the second phone number successfully and keep the original contact intact.</t>
         </is>
       </c>
-      <c r="I24" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J24" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K24" s="1" t="inlineStr">
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Adding a second phone number to an existing contact succeeded and the reply included the new number.</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L24" s="1" t="inlineStr">
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M24" s="1" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N24" s="1" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Validates one-to-many phone-number behavior.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="25" ht="55.2" customHeight="1" s="3">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>TC-024</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>SCN-018</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Return all contacts after data exists</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Verify retrieval of the complete contact list after one or more contacts are present.</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; at least one contact exists.</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; phone_number=12092</t>
         </is>
       </c>
-      <c r="G25" s="1" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create one or more contacts.
@@ -2265,74 +2312,79 @@
 4. Inspect returned list.</t>
         </is>
       </c>
-      <c r="H25" s="1" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>System should return all existing contacts with their phone numbers in a readable logical structure.</t>
         </is>
       </c>
-      <c r="I25" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J25" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K25" s="1" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Retrieving all contacts after data creation returned structured contact data including ali and 12092.</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L25" s="1" t="inlineStr">
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M25" s="1" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N25" s="1" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>Useful baseline for later list assertions.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="26" ht="55.2" customHeight="1" s="3">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>TC-025</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>SCN-019</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Search for an existing contact by name</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Verify retrieval of a contact using its contact name.</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact exists.</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; phone_number=12092</t>
         </is>
       </c>
-      <c r="G26" s="1" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali.
@@ -2340,74 +2392,79 @@
 4. Inspect returned result.</t>
         </is>
       </c>
-      <c r="H26" s="1" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>System should return the matching contact and its stored phone numbers.</t>
         </is>
       </c>
-      <c r="I26" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J26" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K26" s="1" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Searching for an existing contact by name returned the expected contact data.</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L26" s="1" t="inlineStr">
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M26" s="1" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N26" s="1" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Search happy path by name.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="27" ht="55.2" customHeight="1" s="3">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>TC-026</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>SCN-020</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Search for an existing contact by phone number</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>Verify retrieval of a contact using one of its phone numbers.</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact and number exist.</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; phone_number=12092</t>
         </is>
       </c>
-      <c r="G27" s="1" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali with phone number 12092.
@@ -2415,74 +2472,79 @@
 4. Inspect returned result.</t>
         </is>
       </c>
-      <c r="H27" s="1" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>System should return the contact associated with the phone number.</t>
         </is>
       </c>
-      <c r="I27" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J27" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K27" s="1" t="inlineStr">
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Searching for an existing contact by phone number returned the expected contact data.</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L27" s="1" t="inlineStr">
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M27" s="1" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N27" s="1" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>Search happy path by number.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="28" ht="55.2" customHeight="1" s="3">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>TC-027</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>SCN-022</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Edit only the contact name</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Verify successful update of a contact name without changing the phone number.</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact exists.</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>old_name=ali; phone_number=12092; new_name=ali_updated</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali with phone number 12092.
@@ -2490,74 +2552,79 @@
 4. Retrieve the contact by new name.</t>
         </is>
       </c>
-      <c r="H28" s="1" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>System should update the contact name successfully while preserving the phone number.</t>
         </is>
       </c>
-      <c r="I28" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J28" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K28" s="1" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Editing only the contact name succeeded and the updated name remained retrievable with the original phone number.</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L28" s="1" t="inlineStr">
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M28" s="1" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N28" s="1" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Partial update path.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="29" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>TC-028</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>SCN-023</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Edit only the phone number</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Verify successful update of a contact phone number without changing the contact name.</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact exists.</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; old_phone=12092; new_phone=66056477</t>
         </is>
       </c>
-      <c r="G29" s="1" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali with phone number 12092.
@@ -2565,74 +2632,79 @@
 4. Retrieve the contact by name.</t>
         </is>
       </c>
-      <c r="H29" s="1" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>System should update the phone number successfully while preserving the contact name.</t>
         </is>
       </c>
-      <c r="I29" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J29" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K29" s="1" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Editing only the phone number succeeded and the updated number remained retrievable for the same contact.</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L29" s="1" t="inlineStr">
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M29" s="1" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N29" s="1" t="inlineStr">
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>Partial update path for phone values.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="30" ht="68.65000000000001" customHeight="1" s="3">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>TC-029</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>SCN-024</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Edit both contact name and phone number together</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Verify simultaneous update of both contact name and phone number.</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact exists.</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>old_name=ali; old_phone=12092; new_name=ali_updated; new_phone=66056477</t>
         </is>
       </c>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali.
@@ -2640,74 +2712,79 @@
 4. Retrieve contact by new name and/or new number.</t>
         </is>
       </c>
-      <c r="H30" s="1" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>System should update both fields successfully and make the new values searchable.</t>
         </is>
       </c>
-      <c r="I30" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J30" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K30" s="1" t="inlineStr">
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Editing both the contact name and phone number together succeeded and both new values were retrievable.</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L30" s="1" t="inlineStr">
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M30" s="1" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N30" s="1" t="inlineStr">
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>Combined update flow.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+    <row r="31" ht="55.2" customHeight="1" s="3">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>TC-030</t>
         </is>
       </c>
-      <c r="B31" s="1" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>SCN-025</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Delete an existing contact</t>
         </is>
       </c>
-      <c r="D31" s="1" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Verify successful deletion of a known contact.</t>
         </is>
       </c>
-      <c r="E31" s="1" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact exists.</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>contact_name=ali; phone_number=12092</t>
         </is>
       </c>
-      <c r="G31" s="1" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Create contact ali.
@@ -2715,74 +2792,79 @@
 4. Attempt to search for ali afterward.</t>
         </is>
       </c>
-      <c r="H31" s="1" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>System should remove the contact successfully and the contact should no longer be retrievable.</t>
         </is>
       </c>
-      <c r="I31" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J31" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K31" s="1" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Deleting an existing contact and then verifying non-retrievability did not stay controlled; the server stopped during the flow.</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="L31" s="1" t="inlineStr">
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="M31" s="1" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N31" s="1" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>Deletion happy path.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+    <row r="32" ht="55.2" customHeight="1" s="3">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>TC-031</t>
         </is>
       </c>
-      <c r="B32" s="1" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>SCN-021</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Search for a non-existing contact by name</t>
         </is>
       </c>
-      <c r="D32" s="1" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>Verify controlled behavior when searching for a contact name that does not exist.</t>
         </is>
       </c>
-      <c r="E32" s="1" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact does not exist.</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>contact_name=ghost</t>
         </is>
       </c>
-      <c r="G32" s="1" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure target contact ghost does not exist.
@@ -2790,74 +2872,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H32" s="1" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled not-found result without server failure.</t>
         </is>
       </c>
-      <c r="I32" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J32" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K32" s="1" t="inlineStr">
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Searching for a non-existing contact by name did not return a controlled not-found result; the server stopped.</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L32" s="1" t="inlineStr">
+      <c r="M32" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M32" s="1" t="inlineStr">
+      <c r="N32" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N32" s="1" t="inlineStr">
+      <c r="O32" s="4" t="inlineStr">
         <is>
           <t>Wave 2 negative search case.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+    <row r="33" ht="55.2" customHeight="1" s="3">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>TC-032</t>
         </is>
       </c>
-      <c r="B33" s="1" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>SCN-021</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Search for a non-existing contact by phone number</t>
         </is>
       </c>
-      <c r="D33" s="1" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>Verify controlled behavior when searching for a phone number that does not exist.</t>
         </is>
       </c>
-      <c r="E33" s="1" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target phone number does not exist.</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>phone_number=99999999</t>
         </is>
       </c>
-      <c r="G33" s="1" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure target phone number does not exist.
@@ -2865,74 +2952,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H33" s="1" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled not-found result without server failure.</t>
         </is>
       </c>
-      <c r="I33" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J33" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K33" s="1" t="inlineStr">
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Searching for a non-existing contact by phone number did not return a controlled not-found result; the server stopped.</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L33" s="1" t="inlineStr">
+      <c r="M33" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M33" s="1" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N33" s="1" t="inlineStr">
+      <c r="O33" s="4" t="inlineStr">
         <is>
           <t>Wave 2 negative search by number.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="34" ht="55.2" customHeight="1" s="3">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>TC-033</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>SCN-026</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Delete a non-existing contact</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>Verify controlled behavior when removing a contact that does not exist.</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact does not exist.</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>contact_name=ghost</t>
         </is>
       </c>
-      <c r="G34" s="1" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure contact ghost does not exist.
@@ -2940,74 +3032,79 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H34" s="1" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>System should return a predictable controlled outcome without server termination.</t>
         </is>
       </c>
-      <c r="I34" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J34" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K34" s="1" t="inlineStr">
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Removing a non-existing contact returned a misleading success result instead of a controlled not-found outcome.</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L34" s="1" t="inlineStr">
+      <c r="M34" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M34" s="1" t="inlineStr">
+      <c r="N34" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N34" s="1" t="inlineStr">
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>Important to compare delete behavior with other not-found operations.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="35" ht="55.2" customHeight="1" s="3">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>TC-034</t>
         </is>
       </c>
-      <c r="B35" s="1" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>SCN-026</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Edit a non-existing contact</t>
         </is>
       </c>
-      <c r="D35" s="1" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Verify controlled behavior when editing a contact that does not exist.</t>
         </is>
       </c>
-      <c r="E35" s="1" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Server is running; schema initialized; target contact does not exist.</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>old_name=ghost; old_phone=11111; new_name=ghost2; new_phone=22222</t>
         </is>
       </c>
-      <c r="G35" s="1" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>1. Start server.
 2. Ensure contact ghost does not exist.
@@ -3015,43 +3112,124 @@
 4. Observe reply and server stability.</t>
         </is>
       </c>
-      <c r="H35" s="1" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>System should return a controlled not-found outcome without raw internal exception details.</t>
         </is>
       </c>
-      <c r="I35" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="J35" s="1" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="K35" s="1" t="inlineStr">
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Editing a non-existing contact did not return a controlled not-found outcome; the server stopped.</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="L35" s="1" t="inlineStr">
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M35" s="1" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>Automated Candidate</t>
         </is>
       </c>
-      <c r="N35" s="1" t="inlineStr">
+      <c r="O35" s="4" t="inlineStr">
         <is>
           <t>Complements Wave 1 add-number missing-contact case.</t>
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SCN-006</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Reject invalid email format during signup</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Verify that signup rejects malformed email input with a controlled validation result.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Server is running; clean database.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>username=user_bad_email; email=abc; password=1234</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>1. Start server.
+2. Send sign_up with malformed email value abc.
+3. Observe reply and server stability.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>System should reject the invalid email with a structured validation response and keep the server alive.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Malformed email was accepted and signup succeeded instead of returning a controlled validation error.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Automated Candidate</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Added to align the documented case inventory with the implemented invalid-email requirement test.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>